<commit_message>
Yokohama V3.4: pick-up instead of van throughout (D-Max is a pick-up)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015NVtiu1i8y2cgzjuAhfAyB
</commit_message>
<xml_diff>
--- a/09_meetings/Yokohama_2026/ISZE_GPS_Extended_Target_FY27_V3.4.xlsx
+++ b/09_meetings/Yokohama_2026/ISZE_GPS_Extended_Target_FY27_V3.4.xlsx
@@ -839,7 +839,7 @@
     <t xml:space="preserve">LCV / D-Max</t>
   </si>
   <si>
-    <t xml:space="preserve">van rate per vehicle</t>
+    <t xml:space="preserve">pick-up rate per vehicle</t>
   </si>
   <si>
     <t xml:space="preserve">CV LD (N75/N50/N62)</t>
@@ -1196,10 +1196,10 @@
     <t xml:space="preserve">How UIO V19 builds the fleet</t>
   </si>
   <si>
-    <t xml:space="preserve">Up to 2025: registrations of each year, with an age curve for how many vehicles are still on the road. On that curve a van stays on the road about 8 years on average and a truck about 10 years.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">From 2026: the forecast of new van and truck sales is added each year, and only 3% of the fleet leaves the road each year. 3% a year means a vehicle stays on the road about 33 years, so the fleet keeps growing.</t>
+    <t xml:space="preserve">Up to 2025: registrations of each year, with an age curve for how many vehicles are still on the road. On that curve a pick-up stays on the road about 8 years on average and a truck about 10 years.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From 2026: the forecast of new pick-up and truck sales is added each year, and only 3% of the fleet leaves the road each year. 3% a year means a vehicle stays on the road about 33 years, so the fleet keeps growing.</t>
   </si>
   <si>
     <t xml:space="preserve">Result: the fleet of these 18 distributors grows about 26% from FY2026 to FY2031, and the parts potential grows with it.</t>
@@ -1244,31 +1244,31 @@
     <t xml:space="preserve">Medium truck</t>
   </si>
   <si>
-    <t xml:space="preserve">Van (D-Max)</t>
+    <t xml:space="preserve">Pick-up (D-Max)</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
   </si>
   <si>
-    <t xml:space="preserve">of which vans</t>
+    <t xml:space="preserve">of which pick-ups</t>
   </si>
   <si>
     <t xml:space="preserve">of which trucks</t>
   </si>
   <si>
-    <t xml:space="preserve">New vans and vans leaving the road per year (16 distributors and UMI, UIO V19)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vans in use</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vans leaving the road (3% a year)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New vans in the forecast</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New vans = change in vans in use + vans leaving the road. The UIO V20 spec uses the same new vans.</t>
+    <t xml:space="preserve">New pick-ups and pick-ups leaving the road per year (16 distributors and UMI, UIO V19)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick-ups in use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick-ups leaving the road (3% a year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New pick-ups in the forecast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New pick-ups = change in pick-ups in use + pick-ups leaving the road. The UIO V20 spec uses the same new pick-ups.</t>
   </si>
   <si>
     <t xml:space="preserve">Price index (FY2026 = 1)</t>
@@ -1307,16 +1307,16 @@
     <t xml:space="preserve">What is different in the UIO V20 spec</t>
   </si>
   <si>
-    <t xml:space="preserve">Everything up to 2025 is the same as UIO V19, and the forecast of new van and truck sales is the same. Only one thing changes: from 2026 vehicles leave the road on the same age curve as before 2026 (van about 8 years, truck about 10 years) instead of 3% a year.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Effect: each year about 10,000 new vans are added for these distributors, while about 13,000 to 15,000 older vans leave the road. The van fleet therefore goes down instead of up.</t>
+    <t xml:space="preserve">Everything up to 2025 is the same as UIO V19, and the forecast of new pick-up and truck sales is the same. Only one thing changes: from 2026 vehicles leave the road on the same age curve as before 2026 (pick-up about 8 years, truck about 10 years) instead of 3% a year.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Effect: each year about 10,000 new pick-ups are added for these distributors, while about 13,000 to 15,000 older pick-ups leave the road. The pick-up fleet therefore goes down instead of up.</t>
   </si>
   <si>
     <t xml:space="preserve">Medium trucks that UIO V19 shows from 2026 for Ireland, Portugal, Greece and Cyprus are planned vehicles, not registered vehicles; the UIO V20 spec leaves them out. ITUK and UTI are the same in both versions.</t>
   </si>
   <si>
-    <t xml:space="preserve">Our reading: UIO V19 keeps vehicles too long (about 33 years); the UIO V20 curve takes vans off the road early for pick-ups. The real fleet is most likely between the two. The UIO V20 spec is not yet approved, so this file uses UIO V19; this sheet shows what changes if UIO V20 is adopted.</t>
+    <t xml:space="preserve">Our reading: UIO V19 keeps vehicles too long (about 33 years); the UIO V20 curve takes pick-ups off the road early (almost all gone by year 12 to 13). The real fleet is most likely between the two. The UIO V20 spec is not yet approved, so this file uses UIO V19; this sheet shows what changes if UIO V20 is adopted.</t>
   </si>
   <si>
     <t xml:space="preserve">Targets on this sheet: FY2027 stays the same amount (budget + stretch). From FY2028 the same rule as the model: GPS share + the yearly stretch, applied to the smaller UIO V20 potential.</t>
@@ -1689,10 +1689,10 @@
     <t xml:space="preserve">FY31 (+price)</t>
   </si>
   <si>
-    <t xml:space="preserve">ISZE net EUR per van</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Van rate EUR 250 per vehicle (FY2026, ISZE net), +5% in FY2027 = EUR 262.50, then + yearly price input (Dashboard (2) T1). Replaces the earlier EUR 219.56.</t>
+    <t xml:space="preserve">ISZE net EUR per pick-up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick-up rate EUR 250 per vehicle (FY2026, ISZE net), +5% in FY2027 = EUR 262.50, then + yearly price input (Dashboard (2) T1). Replaces the earlier EUR 219.56.</t>
   </si>
   <si>
     <t xml:space="preserve">ISZE -&gt; IUK wholesale (ISZE-net EUR)  &lt;&lt;  EXTENDED TARGET IS SET HERE</t>
@@ -1761,7 +1761,7 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Van rate EUR 250 per vehicle (FY2026, ISZE net), +5% in FY2027 = EUR 262.50. Replaces the earlier EUR 219.56.</t>
+    <t xml:space="preserve">1. Pick-up rate EUR 250 per vehicle (FY2026, ISZE net), +5% in FY2027 = EUR 262.50. Replaces the earlier EUR 219.56.</t>
   </si>
   <si>
     <t xml:space="preserve">UMI — GPS Extended Target FY2027 · UNIVERSAL MOTORS ISRAEL LTD   [LCV only]</t>
@@ -1902,10 +1902,10 @@
     <t xml:space="preserve">F-Series rate</t>
   </si>
   <si>
-    <t xml:space="preserve">Van (D-Max) rate, EUR 250 base</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Truck rates 739 / 887 and van rate EUR 250 per vehicle (FY2026, ISZE net), +5% in FY2027, then + yearly price input. All rates sit on the Inputs sheet.</t>
+    <t xml:space="preserve">Pick-up (D-Max) rate, EUR 250 base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Truck rates 739 / 887 and pick-up rate EUR 250 per vehicle (FY2026, ISZE net), +5% in FY2027, then + yearly price input. All rates sit on the Inputs sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">ISZE -&gt; GERMANY wholesale (ISZE-net EUR)  &lt;&lt;  EXTENDED TARGET IS SET HERE</t>
@@ -1920,7 +1920,7 @@
     <t xml:space="preserve">FY25 11/12 mo · FY26 0/12 mo</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Truck rates 739 / 887 and van rate EUR 250 per vehicle (FY2026, ISZE net), +5% in FY2027, then + yearly price input.</t>
+    <t xml:space="preserve">1. Truck rates 739 / 887 and pick-up rate EUR 250 per vehicle (FY2026, ISZE net), +5% in FY2027, then + yearly price input.</t>
   </si>
   <si>
     <t xml:space="preserve">BELGIUM — GPS Extended Target FY2027 · ISUZU BENELUX NV   [mixed CV+LCV]</t>
@@ -2025,10 +2025,10 @@
     <t xml:space="preserve">1. Parts spend per vehicle (ISZE net, FY2026 base)</t>
   </si>
   <si>
-    <t xml:space="preserve">Van (D-Max) EUR 250. Light truck (LD) EUR 739. Medium truck and F-Series EUR 887. FY2027 +5%, FY2028 to FY2031 +3% a year.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The van rate replaces the earlier EUR 219.56.</t>
+    <t xml:space="preserve">Pick-up (D-Max) EUR 250. Light truck (LD) EUR 739. Medium truck and F-Series EUR 887. FY2027 +5%, FY2028 to FY2031 +3% a year.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The pick-up rate replaces the earlier EUR 219.56.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Vehicles in use</t>
@@ -2107,7 +2107,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Dealer spend per vehicle as in the ITUK row: GBP 400 / 1,000 / 1,200 x 1.12 = EUR 448 (van), 1,120 (light truck), 1,344 (medium truck, F-Series).</t>
+    <t xml:space="preserve">Dealer spend per vehicle as in the ITUK row: GBP 400 / 1,000 / 1,200 x 1.12 = EUR 448 (pick-up), 1,120 (light truck), 1,344 (medium truck, F-Series).</t>
   </si>
   <si>
     <t xml:space="preserve">FY2026 actual = distributor KPI sales to dealers. FY2027 target = FY2026 + ISZE stretch / (1 - 35% distributor margin). FY2028 to FY2031 move with the ISZE target.</t>
@@ -23583,27 +23583,27 @@
         <v>247</v>
       </c>
       <c r="C47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",C12:C45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",C12:C45)</f>
         <v>125140</v>
       </c>
       <c r="D47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",D12:D45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",D12:D45)</f>
         <v>131617</v>
       </c>
       <c r="E47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",E12:E45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",E12:E45)</f>
         <v>137509</v>
       </c>
       <c r="F47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",F12:F45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",F12:F45)</f>
         <v>143079</v>
       </c>
       <c r="G47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",G12:G45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",G12:G45)</f>
         <v>148481</v>
       </c>
       <c r="H47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",H12:H45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",H12:H45)</f>
         <v>153721</v>
       </c>
     </row>
@@ -26734,27 +26734,27 @@
         <v>247</v>
       </c>
       <c r="C47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",C12:C45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",C12:C45)</f>
         <v>125140</v>
       </c>
       <c r="D47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",D12:D45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",D12:D45)</f>
         <v>120562</v>
       </c>
       <c r="E47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",E12:E45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",E12:E45)</f>
         <v>115958</v>
       </c>
       <c r="F47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",F12:F45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",F12:F45)</f>
         <v>111581</v>
       </c>
       <c r="G47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",G12:G45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",G12:G45)</f>
         <v>107656</v>
       </c>
       <c r="H47" s="61" t="n">
-        <f aca="false">SUMIF($B$12:$B$45,"Van (D-Max)",H12:H45)</f>
+        <f aca="false">SUMIF($B$12:$B$45,"Pick-up (D-Max)",H12:H45)</f>
         <v>104185</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Yokohama V3.4: final read-through fixes (labels, coverage notes, ITUK/UTI share wording in mail)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015NVtiu1i8y2cgzjuAhfAyB
</commit_message>
<xml_diff>
--- a/09_meetings/Yokohama_2026/ISZE_GPS_Extended_Target_FY27_V3.4.xlsx
+++ b/09_meetings/Yokohama_2026/ISZE_GPS_Extended_Target_FY27_V3.4.xlsx
@@ -760,7 +760,7 @@
     <t xml:space="preserve">Remaining stretch BEFORE GPS</t>
   </si>
   <si>
-    <t xml:space="preserve">Network BP (PL plan row 186)</t>
+    <t xml:space="preserve">Network plan (BP)</t>
   </si>
   <si>
     <t xml:space="preserve">GPS contribution (18 DBs)</t>
@@ -887,7 +887,7 @@
     <t xml:space="preserve">Fiscal year</t>
   </si>
   <si>
-    <t xml:space="preserve">Network BP, PL plan row 186 (EUR)</t>
+    <t xml:space="preserve">Network plan (BP), EUR</t>
   </si>
   <si>
     <t xml:space="preserve">Sum of BP FY27, 18 distributors</t>
@@ -1406,10 +1406,10 @@
     <t xml:space="preserve">Above 100% at BP: quote the amount, not the %</t>
   </si>
   <si>
-    <t xml:space="preserve">Insufficient data — distributor KPI (IMF/Nordic Auto.) stopped reporting Oct'25, 9 months stale.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Insufficient data — distributor KPI (ISD) stopped reporting Mar'25, 15+ months stale.</t>
+    <t xml:space="preserve">Not enough data: 6 of 12 months reported in FY2026 (KPI file June 2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not enough data: 11 of 12 months in FY2025, none in FY2026 (KPI file June 2026).</t>
   </si>
   <si>
     <t xml:space="preserve">Belgian vehicles only (IBX also serves NL/PL/LU)</t>
@@ -1424,10 +1424,10 @@
     <t xml:space="preserve">Above 100% after stretch: quote the amount, not the %</t>
   </si>
   <si>
-    <t xml:space="preserve">Insufficient data — Petros Petropoulos stale since Jun'25 (12+ months).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Insufficient data — Cyprus's real distributor (Loutsios &amp; Sons) has zero KPI data. KPI's 'MIDI' row is Italy's, not Cyprus's — excluded.</t>
+    <t xml:space="preserve">Not enough data: 8 of 12 months in FY2025, none in FY2026 (KPI file June 2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not enough data: no KPI figures from Loutsios &amp; Sons.</t>
   </si>
   <si>
     <r>
@@ -1719,7 +1719,7 @@
     <t xml:space="preserve">Share (GPS, ISZE level)</t>
   </si>
   <si>
-    <t xml:space="preserve">Stretch (%) = global input, capped at ceiling</t>
+    <t xml:space="preserve">Stretch (%) = global input (capped only if Dashboard (2) Q1 = YES)</t>
   </si>
   <si>
     <t xml:space="preserve">Stretch amount (= max spend x stretch%)</t>

</xml_diff>